<commit_message>
Pipline con olimpica y farmatodo
</commit_message>
<xml_diff>
--- a/Template_HRC.xlsx
+++ b/Template_HRC.xlsx
@@ -612,7 +612,11 @@
       <c r="H19" s="2" t="n">
         <v>31277975</v>
       </c>
-      <c r="I19" s="7" t="inlineStr"/>
+      <c r="I19" s="7" t="inlineStr">
+        <is>
+          <t xml:space="preserve"> PMP1249244</t>
+        </is>
+      </c>
     </row>
     <row r="20">
       <c r="C20" s="6" t="inlineStr">
@@ -633,7 +637,11 @@
       <c r="H20" s="2" t="n">
         <v>1102345</v>
       </c>
-      <c r="I20" s="7" t="inlineStr"/>
+      <c r="I20" s="7" t="inlineStr">
+        <is>
+          <t xml:space="preserve"> PMP1249258</t>
+        </is>
+      </c>
     </row>
     <row r="21">
       <c r="C21" s="6" t="inlineStr">
@@ -654,7 +662,11 @@
       <c r="H21" s="2" t="n">
         <v>27692682</v>
       </c>
-      <c r="I21" s="7" t="inlineStr"/>
+      <c r="I21" s="7" t="inlineStr">
+        <is>
+          <t xml:space="preserve"> PMP1249400</t>
+        </is>
+      </c>
     </row>
     <row r="22">
       <c r="C22" s="6" t="inlineStr">
@@ -675,7 +687,11 @@
       <c r="H22" s="2" t="n">
         <v>4992313</v>
       </c>
-      <c r="I22" s="7" t="inlineStr"/>
+      <c r="I22" s="7" t="inlineStr">
+        <is>
+          <t xml:space="preserve"> PMP1249405</t>
+        </is>
+      </c>
     </row>
     <row r="23">
       <c r="C23" s="6" t="inlineStr">
@@ -696,7 +712,11 @@
       <c r="H23" s="2" t="n">
         <v>20100423</v>
       </c>
-      <c r="I23" s="7" t="inlineStr"/>
+      <c r="I23" s="7" t="inlineStr">
+        <is>
+          <t xml:space="preserve"> PMP1249557</t>
+        </is>
+      </c>
     </row>
     <row r="24">
       <c r="C24" s="6" t="inlineStr">
@@ -717,7 +737,11 @@
       <c r="H24" s="2" t="n">
         <v>72307698</v>
       </c>
-      <c r="I24" s="7" t="inlineStr"/>
+      <c r="I24" s="7" t="inlineStr">
+        <is>
+          <t xml:space="preserve"> PMP1249558</t>
+        </is>
+      </c>
     </row>
     <row r="25">
       <c r="C25" s="6" t="inlineStr">
@@ -738,7 +762,11 @@
       <c r="H25" s="2" t="n">
         <v>94379986</v>
       </c>
-      <c r="I25" s="7" t="inlineStr"/>
+      <c r="I25" s="7" t="inlineStr">
+        <is>
+          <t xml:space="preserve"> PMP1249559</t>
+        </is>
+      </c>
     </row>
     <row r="26">
       <c r="C26" s="6" t="inlineStr">
@@ -759,7 +787,11 @@
       <c r="H26" s="2" t="n">
         <v>2263380</v>
       </c>
-      <c r="I26" s="7" t="inlineStr"/>
+      <c r="I26" s="7" t="inlineStr">
+        <is>
+          <t xml:space="preserve"> PMP1249560</t>
+        </is>
+      </c>
     </row>
     <row r="27">
       <c r="C27" s="6" t="inlineStr">
@@ -780,7 +812,11 @@
       <c r="H27" s="2" t="n">
         <v>79954317</v>
       </c>
-      <c r="I27" s="7" t="inlineStr"/>
+      <c r="I27" s="7" t="inlineStr">
+        <is>
+          <t xml:space="preserve"> PMP1249561</t>
+        </is>
+      </c>
     </row>
     <row r="28">
       <c r="C28" s="6" t="inlineStr">
@@ -801,7 +837,11 @@
       <c r="H28" s="2" t="n">
         <v>19480076</v>
       </c>
-      <c r="I28" s="7" t="inlineStr"/>
+      <c r="I28" s="7" t="inlineStr">
+        <is>
+          <t xml:space="preserve"> PMP1249562</t>
+        </is>
+      </c>
     </row>
     <row r="29">
       <c r="C29" s="6" t="inlineStr">
@@ -822,7 +862,11 @@
       <c r="H29" s="2" t="n">
         <v>122200697</v>
       </c>
-      <c r="I29" s="7" t="inlineStr"/>
+      <c r="I29" s="7" t="inlineStr">
+        <is>
+          <t xml:space="preserve"> PMP1249563</t>
+        </is>
+      </c>
     </row>
     <row r="30">
       <c r="C30" s="6" t="inlineStr">
@@ -843,7 +887,11 @@
       <c r="H30" s="2" t="n">
         <v>7344450</v>
       </c>
-      <c r="I30" s="7" t="inlineStr"/>
+      <c r="I30" s="7" t="inlineStr">
+        <is>
+          <t xml:space="preserve"> PMP1249564</t>
+        </is>
+      </c>
     </row>
     <row r="31">
       <c r="C31" s="6" t="inlineStr">
@@ -864,7 +912,11 @@
       <c r="H31" s="2" t="n">
         <v>75077367</v>
       </c>
-      <c r="I31" s="7" t="inlineStr"/>
+      <c r="I31" s="7" t="inlineStr">
+        <is>
+          <t xml:space="preserve"> PMP1249565</t>
+        </is>
+      </c>
     </row>
     <row r="32">
       <c r="C32" s="6" t="inlineStr">
@@ -885,7 +937,11 @@
       <c r="H32" s="2" t="n">
         <v>15478421</v>
       </c>
-      <c r="I32" s="7" t="inlineStr"/>
+      <c r="I32" s="7" t="inlineStr">
+        <is>
+          <t xml:space="preserve"> PMP1249566</t>
+        </is>
+      </c>
     </row>
     <row r="33">
       <c r="C33" s="6" t="inlineStr">
@@ -906,7 +962,11 @@
       <c r="H33" s="2" t="n">
         <v>5509234</v>
       </c>
-      <c r="I33" s="7" t="inlineStr"/>
+      <c r="I33" s="7" t="inlineStr">
+        <is>
+          <t xml:space="preserve"> PMP1249894</t>
+        </is>
+      </c>
     </row>
     <row r="34">
       <c r="C34" s="6" t="inlineStr">
@@ -927,7 +987,11 @@
       <c r="H34" s="2" t="n">
         <v>11607265</v>
       </c>
-      <c r="I34" s="7" t="inlineStr"/>
+      <c r="I34" s="7" t="inlineStr">
+        <is>
+          <t xml:space="preserve"> PMP1249897</t>
+        </is>
+      </c>
     </row>
     <row r="35">
       <c r="C35" s="6" t="inlineStr">
@@ -948,7 +1012,11 @@
       <c r="H35" s="2" t="n">
         <v>3747972</v>
       </c>
-      <c r="I35" s="7" t="inlineStr"/>
+      <c r="I35" s="7" t="inlineStr">
+        <is>
+          <t xml:space="preserve"> PMP1249898</t>
+        </is>
+      </c>
     </row>
     <row r="36">
       <c r="C36" s="6" t="inlineStr">
@@ -969,7 +1037,11 @@
       <c r="H36" s="2" t="n">
         <v>1322814</v>
       </c>
-      <c r="I36" s="7" t="inlineStr"/>
+      <c r="I36" s="7" t="inlineStr">
+        <is>
+          <t xml:space="preserve"> PMP1249901</t>
+        </is>
+      </c>
     </row>
     <row r="37">
       <c r="C37" s="6" t="inlineStr">
@@ -990,7 +1062,11 @@
       <c r="H37" s="2" t="n">
         <v>125839982</v>
       </c>
-      <c r="I37" s="7" t="inlineStr"/>
+      <c r="I37" s="7" t="inlineStr">
+        <is>
+          <t xml:space="preserve"> PMP1249972</t>
+        </is>
+      </c>
     </row>
     <row r="38">
       <c r="C38" s="6" t="inlineStr">
@@ -1011,7 +1087,11 @@
       <c r="H38" s="2" t="n">
         <v>28730082</v>
       </c>
-      <c r="I38" s="7" t="inlineStr"/>
+      <c r="I38" s="7" t="inlineStr">
+        <is>
+          <t xml:space="preserve"> PMP1249973</t>
+        </is>
+      </c>
     </row>
     <row r="39">
       <c r="C39" s="6" t="inlineStr">
@@ -1032,7 +1112,11 @@
       <c r="H39" s="2" t="n">
         <v>3055563</v>
       </c>
-      <c r="I39" s="7" t="inlineStr"/>
+      <c r="I39" s="7" t="inlineStr">
+        <is>
+          <t xml:space="preserve"> PMP1249974</t>
+        </is>
+      </c>
     </row>
     <row r="40">
       <c r="C40" s="6" t="inlineStr">
@@ -1053,7 +1137,11 @@
       <c r="H40" s="2" t="n">
         <v>198843616</v>
       </c>
-      <c r="I40" s="7" t="inlineStr"/>
+      <c r="I40" s="7" t="inlineStr">
+        <is>
+          <t xml:space="preserve"> PMP1249975</t>
+        </is>
+      </c>
     </row>
     <row r="41">
       <c r="C41" s="6" t="inlineStr">
@@ -1074,7 +1162,11 @@
       <c r="H41" s="2" t="n">
         <v>86264216</v>
       </c>
-      <c r="I41" s="7" t="inlineStr"/>
+      <c r="I41" s="7" t="inlineStr">
+        <is>
+          <t xml:space="preserve"> PMP1249976</t>
+        </is>
+      </c>
     </row>
     <row r="42">
       <c r="C42" s="6" t="inlineStr">
@@ -1095,7 +1187,11 @@
       <c r="H42" s="2" t="n">
         <v>62919991</v>
       </c>
-      <c r="I42" s="7" t="inlineStr"/>
+      <c r="I42" s="7" t="inlineStr">
+        <is>
+          <t xml:space="preserve"> PMP1250219</t>
+        </is>
+      </c>
     </row>
     <row r="43">
       <c r="C43" s="6" t="inlineStr">
@@ -1116,7 +1212,11 @@
       <c r="H43" s="2" t="n">
         <v>2602887</v>
       </c>
-      <c r="I43" s="7" t="inlineStr"/>
+      <c r="I43" s="7" t="inlineStr">
+        <is>
+          <t xml:space="preserve"> PMP1250222</t>
+        </is>
+      </c>
     </row>
     <row r="44">
       <c r="C44" s="6" t="inlineStr">
@@ -1137,7 +1237,11 @@
       <c r="H44" s="2" t="n">
         <v>39567495</v>
       </c>
-      <c r="I44" s="7" t="inlineStr"/>
+      <c r="I44" s="7" t="inlineStr">
+        <is>
+          <t xml:space="preserve"> PMP1250223</t>
+        </is>
+      </c>
     </row>
     <row r="45">
       <c r="C45" s="6" t="inlineStr">
@@ -1158,7 +1262,11 @@
       <c r="H45" s="2" t="n">
         <v>10928542</v>
       </c>
-      <c r="I45" s="7" t="inlineStr"/>
+      <c r="I45" s="7" t="inlineStr">
+        <is>
+          <t xml:space="preserve"> PMP1250224</t>
+        </is>
+      </c>
     </row>
     <row r="46">
       <c r="C46" s="6" t="inlineStr">
@@ -1179,7 +1287,11 @@
       <c r="H46" s="2" t="n">
         <v>34995137</v>
       </c>
-      <c r="I46" s="7" t="inlineStr"/>
+      <c r="I46" s="7" t="inlineStr">
+        <is>
+          <t xml:space="preserve"> PMP1250225</t>
+        </is>
+      </c>
     </row>
     <row r="47">
       <c r="C47" s="6" t="inlineStr">

</xml_diff>